<commit_message>
v3.4.1 — Multi-sheet aware user preferences
✨ Added
- Each worksheet now maintains its own validation and duplicate-policy preferences.
- Preferences JSON upgraded to include per-sheet sections under sheets.
- Automatically restores the correct settings per sheet on load or switch.

💡 Improved
- Eliminates overwriting when saving multi-sheet workbooks.
- Maintains backward compatibility with older .prefs.json structures.

🧠 Technical
- Refactored _save_user_prefs() and _load_user_prefs() for sheet-aware persistence.
</commit_message>
<xml_diff>
--- a/sample_template.xlsx
+++ b/sample_template.xlsx
@@ -3,22 +3,21 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8130" yWindow="2115" windowWidth="20670" windowHeight="13365" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="with_formulas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -57,11 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,7 +438,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E75"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="16.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -756,7 +754,7 @@
           <t>Employed</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="2" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -1983,7 +1981,7 @@
           <t>afds</t>
         </is>
       </c>
-      <c r="E73" s="3" t="n">
+      <c r="E73" s="2" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -2006,7 +2004,7 @@
           <t>asdf</t>
         </is>
       </c>
-      <c r="E74" s="3" t="n">
+      <c r="E74" s="2" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -2026,7 +2024,7 @@
           <t>asdfasdf</t>
         </is>
       </c>
-      <c r="E75" s="3" t="n">
+      <c r="E75" s="2" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -2042,7 +2040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2061,6 +2059,31 @@
           <t>sum_salary</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>test name 111</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>af</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
corrected variable resulting to not saving prefs per-sheet
</commit_message>
<xml_diff>
--- a/sample_template.xlsx
+++ b/sample_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8130" yWindow="2115" windowWidth="20670" windowHeight="13365" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1950" yWindow="1950" windowWidth="20670" windowHeight="13365" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -437,8 +437,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="16.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -555,7 +555,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Emily Chen</t>
+          <t>Emily Chenssss</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -570,6 +570,9 @@
         <is>
           <t>Unemployed</t>
         </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>45870</v>
       </c>
     </row>
     <row r="7">
@@ -2026,6 +2029,29 @@
       </c>
       <c r="E75" s="2" t="n">
         <v>45658</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>aaaa</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>aaaaa</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>45870</v>
       </c>
     </row>
   </sheetData>
@@ -2040,7 +2066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2085,6 +2111,46 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>aaaa</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>prefs</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
working on visual cues for numeric-value-containing cells. implemented 'indicator', getting issues on _on_tree_hover() --- test to see console error,
</commit_message>
<xml_diff>
--- a/sample_template.xlsx
+++ b/sample_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1950" yWindow="1950" windowWidth="20670" windowHeight="13365" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -56,10 +56,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,12 +438,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:E77"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="16.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="16.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="30.5703125" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
+    <col width="16.42578125" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
+    <col width="16.7109375" bestFit="1" customWidth="1" style="3" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,7 +454,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Age</t>
+          <t>price</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -499,7 +500,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45</v>
+        <v>45.52</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -510,6 +511,9 @@
         <is>
           <t>Employed</t>
         </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>45975</v>
       </c>
     </row>
     <row r="4">
@@ -539,7 +543,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28</v>
+        <v>28.222</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1622,10 +1626,8 @@
           <t>teppy</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
+      <c r="B59" t="n">
+        <v>44</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1644,10 +1646,8 @@
           <t>another</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="B60" t="n">
+        <v>33</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1755,20 +1755,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B65" t="n">
+        <v>12</v>
+      </c>
+      <c r="C65" t="n">
+        <v>12</v>
+      </c>
+      <c r="D65" t="n">
+        <v>2</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1782,20 +1776,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="B66" t="n">
+        <v>11</v>
+      </c>
+      <c r="C66" t="n">
+        <v>12</v>
+      </c>
+      <c r="D66" t="n">
+        <v>12</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1809,20 +1797,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="B67" t="n">
+        <v>12</v>
+      </c>
+      <c r="C67" t="n">
+        <v>12</v>
+      </c>
+      <c r="D67" t="n">
+        <v>12</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1836,20 +1818,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="B68" t="n">
+        <v>12</v>
+      </c>
+      <c r="C68" t="n">
+        <v>12</v>
+      </c>
+      <c r="D68" t="n">
+        <v>12</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1863,20 +1839,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="B69" t="n">
+        <v>12</v>
+      </c>
+      <c r="C69" t="n">
+        <v>12</v>
+      </c>
+      <c r="D69" t="n">
+        <v>12</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1890,20 +1860,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>1</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -1917,20 +1881,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -1944,20 +1902,14 @@
           <t>jane doe</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B72" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" t="n">
+        <v>2</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2017,6 +1969,9 @@
           <t>patrick</t>
         </is>
       </c>
+      <c r="B75" t="n">
+        <v>445.4555</v>
+      </c>
       <c r="C75" t="inlineStr">
         <is>
           <t>aadsf</t>
@@ -2052,6 +2007,21 @@
       </c>
       <c r="E76" s="2" t="n">
         <v>45870</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>asdf</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>12.222</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2066,7 +2036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2102,7 +2072,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>af</t>
+          <t>1231.3333333</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2148,6 +2118,26 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fffsdf</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12.22222</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>15222.5555</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>test</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
uploading backup version from gemini
</commit_message>
<xml_diff>
--- a/sample_template.xlsx
+++ b/sample_template.xlsx
@@ -438,8 +438,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E78"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30.5703125" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="16.42578125" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
@@ -2021,6 +2021,26 @@
       <c r="C77" t="inlineStr">
         <is>
           <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>asdf</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>12.222</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
     </row>

</xml_diff>